<commit_message>
feat(v2 UI): feature Cohort discovery near top of left nav
The cohort board tells the whole v2 story (per-patient -> corpus-level), so it
belongs right under the home harness, not buried second-from-bottom. Rulebook
RoutingAndNavigation: admin.cohort SortOrder 95 -> 91.5 (directly under
admin.harness=91), DisplayName 'Cohort' -> 'Cohort discovery'. Build regenerates
the routing view; SortOrder/DisplayName are raw cols on a pre-existing row so the
ON-CONFLICT reseed clobber is handled in the 05b-customize-data.sql seam (force
UPDATE), keeping a reseeded DB in sync with the hub. Verified live: nav now reads
Harness -> Cohort discovery -> Routing.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/xlsx/causal-autoimmune-architecture-platform.xlsx
+++ b/xlsx/causal-autoimmune-architecture-platform.xlsx
@@ -11309,7 +11309,7 @@
     <t>nav-admin-cohort</t>
   </si>
   <si>
-    <t>Cohort</t>
+    <t>Cohort discovery</t>
   </si>
   <si>
     <t>/admin/cohort</t>
@@ -21522,10 +21522,10 @@
       },
       {
         "RoutingAndNavigationId": "nav-admin-cohort",
-        "DisplayName": "Cohort",
+        "DisplayName": "Cohort discovery",
         "Route": "/admin/cohort",
         "Description": "All 7 cases and their keystone verdicts.",
-        "SortOrder": 95,
+        "SortOrder": 91.5,
         "ParentRouteKey": "admin",
         "RouteKey": "admin.cohort",
         "NavLevel": "sub",
@@ -22385,10 +22385,10 @@
         "ToState": "diagnosis-lifecycle--notactionable",
         "GuardDescription": "Cryptic-relatedness leakage \u21d2 HasSpuriousCorrelationFlag.",
         "TriggeredByRole": "system",
-        "CreatedBy":</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> "build-seed",
+        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">"CreatedBy": "build-seed",
         "ModifiedBy": "build-seed",
         "Name": "diagnosis-lifecycle--mechanismconfirmed-&gt;notactionable",
         "RelativePath": "/admin/state-machine/rules/diagnosis-lifecycle--mechanismconfirmed-&gt;notactionable",
@@ -23183,10 +23183,10 @@
         "ToStateKey": "Actionable",
         "TransitionAt": "2026-06-06T09:00:00Z",
         "TriggeredByRole": "system",
-        "Reason": "transport passes \u2014 actionable de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spite holdout.",
+        "Reason": "transport passes \u2014 a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ctionable despite holdout.",
         "CreatedBy": "build-seed",
         "ModifiedBy": "build-seed",
         "Name": "st-g-06-transportchecked-to-actionable",
@@ -24008,10 +24008,10 @@
         "CreatedBy": "build-seed",
         "ModifiedBy": "build-seed",
         "Name": "ssi-pred-d-notactionable-4",
-        "RelativePath": "/admin/stat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">e-machine/instances/ssi-pred-d-notactionable-4",
+        "RelativePath": </t>
+  </si>
+  <si>
+    <t xml:space="preserve">"/admin/state-machine/instances/ssi-pred-d-notactionable-4",
         "IsCurrent": true,
         "HasCompleteLineage": true,
         "CreatedAt": null,
@@ -24780,10 +24780,10 @@
       },
       {
         "MetaKey": "band.temperature.fever-high",
-        "Category": "ba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nd-threshold",
+        "Ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tegory": "band-threshold",
         "Value": "100.5",
         "ValueType": "number",
         "Description": "Upper bound (degF) of the 'light fever' band; strictly above this is a 'severe fever'.",
@@ -25554,10 +25554,10 @@
         "ComplementC3": 70,
         "ComplementC4": 10,
         "ProteinuriaGPerDay": 0.3,
-        "EgfrMlMin":</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 90,
+        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">"EgfrMlMin": 90,
         "HasActiveUrinarySediment": false,
         "PriorObservation": "sero-ind-c-chen-1",
         "Name": "sero-ind-c-chen-2",
@@ -40855,7 +40855,7 @@
       </c>
       <c r="B23" s="3" t="str">
         <f>SUBSTITUTE(LOWER(C23), " ", "-")</f>
-        <v>cohort</v>
+        <v>cohort-discovery</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>1086</v>
@@ -40867,7 +40867,7 @@
         <v>1088</v>
       </c>
       <c r="F23" s="2">
-        <v>95</v>
+        <v>91.5</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>1055</v>

</xml_diff>